<commit_message>
fix: retain native image copy errors through controlled shared maintenance
</commit_message>
<xml_diff>
--- a/outputs/meituan-waimai-negative-review-appeals-20261028/美团外卖差评申诉汇总-2026-10-27.xlsx
+++ b/outputs/meituan-waimai-negative-review-appeals-20261028/美团外卖差评申诉汇总-2026-10-27.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="申诉汇总" sheetId="1" r:id="Rba00cfa78e6c450e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="申诉汇总" sheetId="1" r:id="R59bbfcca75bd479d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2829,7 +2829,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe6a388f843b4f91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2f7bc24d1184de7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: classify image-only product pages and stop replaying submitted appeal closings
</commit_message>
<xml_diff>
--- a/outputs/meituan-waimai-negative-review-appeals-20261028/美团外卖差评申诉汇总-2026-10-27.xlsx
+++ b/outputs/meituan-waimai-negative-review-appeals-20261028/美团外卖差评申诉汇总-2026-10-27.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="申诉汇总" sheetId="1" r:id="R59bbfcca75bd479d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="申诉汇总" sheetId="1" r:id="R7595a7fcd1044575"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -406,13 +406,13 @@
         <x:v>申诉中</x:v>
       </x:c>
       <x:c r="H5" s="7" t="n">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="I5" s="7" t="str">
         <x:v>未申诉</x:v>
       </x:c>
       <x:c r="J5" s="7" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2771,10 +2771,10 @@
         <x:v>这米饭是放了多久了，加了咖喱泡了一会儿都硬的一批</x:v>
       </x:c>
       <x:c r="F74" s="17" t="str">
-        <x:v>预申述语句</x:v>
+        <x:v>AI申诉</x:v>
       </x:c>
       <x:c r="G74" s="17" t="str">
-        <x:v>未读取</x:v>
+        <x:v>申诉时间:2026-10-28 18:40:53</x:v>
       </x:c>
       <x:c r="H74" s="17" t="str">
         <x:v>自动申诉已关闭</x:v>
@@ -2829,7 +2829,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2f7bc24d1184de7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ab6bd438dc64e3c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>